<commit_message>
Refresh 2026-2027 fee and payment data
Updated the 2026-2027 fee workbook and student term ledger to reflect revised fee totals, payments, and outstanding balances for multiple students. This also includes parent code sheet updates to keep the reference data aligned with the current records.
</commit_message>
<xml_diff>
--- a/2026 - 2027 FEE.xlsx
+++ b/2026 - 2027 FEE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11F32D7-9D41-4AE4-AC61-9359E3DBF28A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A39421B-28DF-4BA5-994C-6BB39D92F96B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1ST TERM ACCOUNT" sheetId="14" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="308">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -953,6 +953,15 @@
   <si>
     <t>ABDULAZEEZ FAMILY</t>
   </si>
+  <si>
+    <t>NIP:PAUL ADEDOJA</t>
+  </si>
+  <si>
+    <t>ISLAMIAT YETUNDE TIRIMISIYU</t>
+  </si>
+  <si>
+    <t>ADIGUN AHNAF</t>
+  </si>
 </sst>
 </file>
 
@@ -2136,7 +2145,7 @@
         <v>44</v>
       </c>
       <c r="D7" s="23">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="E7" s="24">
         <v>0</v>
@@ -2159,7 +2168,7 @@
       </c>
       <c r="K7" s="24">
         <f t="shared" si="1"/>
-        <v>18200</v>
+        <v>19500</v>
       </c>
       <c r="L7" s="24">
         <f t="shared" si="2"/>
@@ -2208,14 +2217,14 @@
       </c>
       <c r="Z7" s="24">
         <f t="shared" si="5"/>
-        <v>43130</v>
+        <v>44430</v>
       </c>
       <c r="AA7" s="24">
-        <v>43130</v>
+        <v>20000</v>
       </c>
       <c r="AB7" s="20">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>24430</v>
       </c>
       <c r="AC7" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2231,7 +2240,7 @@
       </c>
       <c r="AF7" s="25" t="str">
         <f t="shared" si="10"/>
-        <v>BONUS</v>
+        <v/>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
@@ -2429,11 +2438,11 @@
         <v>44280</v>
       </c>
       <c r="AA9" s="24">
-        <v>16870</v>
+        <v>20000</v>
       </c>
       <c r="AB9" s="20">
         <f t="shared" si="6"/>
-        <v>27410</v>
+        <v>24280</v>
       </c>
       <c r="AC9" s="24" t="str">
         <f t="shared" si="7"/>
@@ -2538,11 +2547,11 @@
         <v>69290</v>
       </c>
       <c r="AA10" s="24">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="AB10" s="20">
         <f t="shared" si="6"/>
-        <v>69290</v>
+        <v>49290</v>
       </c>
       <c r="AC10" s="24" t="str">
         <f t="shared" si="7"/>
@@ -3444,7 +3453,7 @@
         <v>33</v>
       </c>
       <c r="D19" s="23">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E19" s="24">
         <v>0</v>
@@ -3467,7 +3476,7 @@
       </c>
       <c r="K19" s="24">
         <f t="shared" si="1"/>
-        <v>21000</v>
+        <v>19600</v>
       </c>
       <c r="L19" s="24">
         <f t="shared" si="2"/>
@@ -3475,11 +3484,11 @@
       </c>
       <c r="M19" s="24">
         <f t="shared" si="3"/>
-        <v>1875</v>
+        <v>1750</v>
       </c>
       <c r="N19" s="24">
         <f t="shared" si="4"/>
-        <v>3750</v>
+        <v>3500</v>
       </c>
       <c r="O19" s="24">
         <v>25970</v>
@@ -3516,18 +3525,18 @@
       </c>
       <c r="Z19" s="24">
         <f t="shared" si="5"/>
-        <v>73925</v>
+        <v>72150</v>
       </c>
       <c r="AA19" s="24">
-        <v>51685</v>
+        <v>72150</v>
       </c>
       <c r="AB19" s="20">
         <f t="shared" si="6"/>
-        <v>22240</v>
-      </c>
-      <c r="AC19" s="24" t="str">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="24">
         <f t="shared" si="7"/>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="AD19" s="24" t="str">
         <f t="shared" si="8"/>
@@ -3539,7 +3548,7 @@
       </c>
       <c r="AF19" s="25" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>BONUS</v>
       </c>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.25">
@@ -3628,11 +3637,11 @@
         <v>76770</v>
       </c>
       <c r="AA20" s="24">
-        <v>0</v>
+        <v>9535</v>
       </c>
       <c r="AB20" s="20">
         <f t="shared" si="6"/>
-        <v>76770</v>
+        <v>67235</v>
       </c>
       <c r="AC20" s="24" t="str">
         <f t="shared" si="7"/>
@@ -4752,7 +4761,7 @@
         <v>49</v>
       </c>
       <c r="D31" s="23">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="E31" s="24">
         <v>0</v>
@@ -4775,7 +4784,7 @@
       </c>
       <c r="K31" s="24">
         <f t="shared" si="1"/>
-        <v>26000</v>
+        <v>24700</v>
       </c>
       <c r="L31" s="24">
         <f t="shared" si="2"/>
@@ -4783,7 +4792,7 @@
       </c>
       <c r="M31" s="24">
         <f t="shared" si="3"/>
-        <v>1000</v>
+        <v>950</v>
       </c>
       <c r="N31" s="24">
         <f t="shared" si="4"/>
@@ -4824,14 +4833,14 @@
       </c>
       <c r="Z31" s="24">
         <f t="shared" si="5"/>
+        <v>41790</v>
+      </c>
+      <c r="AA31" s="24">
         <v>43140</v>
-      </c>
-      <c r="AA31" s="24">
-        <v>0</v>
       </c>
       <c r="AB31" s="20">
         <f t="shared" si="6"/>
-        <v>43140</v>
+        <v>-1350</v>
       </c>
       <c r="AC31" s="24" t="str">
         <f t="shared" si="7"/>
@@ -4847,7 +4856,7 @@
       </c>
       <c r="AF31" s="25" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>BONUS</v>
       </c>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.25">
@@ -12120,14 +12129,14 @@
         <v>0</v>
       </c>
       <c r="Z98" s="24">
-        <f t="shared" ref="Z98:Z129" si="37">SUM(J98:Y98)</f>
+        <f t="shared" ref="Z98:Z124" si="37">SUM(J98:Y98)</f>
         <v>73925</v>
       </c>
       <c r="AA98" s="24">
         <v>0</v>
       </c>
       <c r="AB98" s="20">
-        <f t="shared" ref="AB98:AB129" si="38">Z98-AA98</f>
+        <f t="shared" ref="AB98:AB124" si="38">Z98-AA98</f>
         <v>73925</v>
       </c>
       <c r="AC98" s="24" t="str">
@@ -14996,8 +15005,8 @@
       <c r="L125" s="28"/>
       <c r="M125" s="28"/>
       <c r="N125" s="28">
-        <f t="shared" ref="N125:AF125" si="42">SUM(N2:N124)</f>
-        <v>259500</v>
+        <f t="shared" ref="N125:AE125" si="42">SUM(N2:N124)</f>
+        <v>259250</v>
       </c>
       <c r="O125" s="28">
         <f t="shared" si="42"/>
@@ -15045,19 +15054,19 @@
       </c>
       <c r="Z125" s="28">
         <f t="shared" si="42"/>
-        <v>7613565</v>
+        <v>7611740</v>
       </c>
       <c r="AA125" s="28">
         <f t="shared" si="42"/>
-        <v>1291035</v>
+        <v>1364175</v>
       </c>
       <c r="AB125" s="28">
         <f t="shared" si="42"/>
-        <v>6322530</v>
+        <v>6247565</v>
       </c>
       <c r="AC125" s="28">
         <f t="shared" si="42"/>
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="AD125" s="28">
         <f t="shared" si="42"/>
@@ -23308,7 +23317,7 @@
       </c>
       <c r="F1" s="36">
         <f>SUM(D2:D1000)</f>
-        <v>1291035</v>
+        <v>1364175</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
@@ -24130,10 +24139,21 @@
       <c r="X29" s="7"/>
     </row>
     <row r="30" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="7"/>
+      <c r="A30" s="8">
+        <v>46278</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="D30" s="9">
+        <v>30000</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>254</v>
+      </c>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
@@ -24155,10 +24175,21 @@
       <c r="X30" s="7"/>
     </row>
     <row r="31" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="7"/>
+      <c r="A31" s="8">
+        <v>46278</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="D31" s="9">
+        <v>43140</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>307</v>
+      </c>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
@@ -38184,17 +38215,17 @@
       </c>
       <c r="B2" s="15">
         <f>'1ST TERM ACCOUNT'!AC125</f>
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="C2" s="15">
         <f>B2*0.7</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
       <c r="D2" s="15"/>
       <c r="E2" s="16"/>
       <c r="F2" s="15">
         <f>$C$2-D2</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -38210,7 +38241,7 @@
       <c r="E3" s="16"/>
       <c r="F3" s="15">
         <f>$C$2-(D2+D3)</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -38219,14 +38250,14 @@
       </c>
       <c r="B4" s="15">
         <f>B3-B2</f>
-        <v>204000</v>
+        <v>198000</v>
       </c>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="16"/>
       <c r="F4" s="15">
         <f>$C$2-(D2+D3+D4)</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -38236,7 +38267,7 @@
       <c r="E5" s="16"/>
       <c r="F5" s="15">
         <f>$C$2-(D2+D3+D4+D5)</f>
-        <v>8400</v>
+        <v>12600</v>
       </c>
       <c r="H5" s="17"/>
     </row>

</xml_diff>

<commit_message>
Correct fee data and class names
This change updates the student fee dataset to fix a mis-typed class name and correct several payment and balance entries in the 2026–2027 fee records. It also syncs the related Excel files and student JSON data with the latest verified totals for the affected students.
</commit_message>
<xml_diff>
--- a/2026 - 2027 FEE.xlsx
+++ b/2026 - 2027 FEE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{509D76EA-8349-4561-BD0A-BCB99C049F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F37F3DD-24FE-4729-8069-F8D7965C8870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="406">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -1200,9 +1200,6 @@
     <t>TESTIMONY AYANFE</t>
   </si>
   <si>
-    <t>PRINARY 2</t>
-  </si>
-  <si>
     <t>OLADOSU</t>
   </si>
   <si>
@@ -1252,6 +1249,12 @@
   </si>
   <si>
     <t>MOSES HEPHZIBAH</t>
+  </si>
+  <si>
+    <t>OFURE DIVINE EDIALE</t>
+  </si>
+  <si>
+    <t>OSIGWE FAMILY</t>
   </si>
 </sst>
 </file>
@@ -6089,10 +6092,10 @@
     </row>
     <row r="41" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A41" s="22" t="s">
+        <v>389</v>
+      </c>
+      <c r="B41" s="22" t="s">
         <v>390</v>
-      </c>
-      <c r="B41" s="22" t="s">
-        <v>391</v>
       </c>
       <c r="C41" s="22" t="s">
         <v>44</v>
@@ -9320,7 +9323,7 @@
         <v>368</v>
       </c>
       <c r="C71" s="22" t="s">
-        <v>387</v>
+        <v>48</v>
       </c>
       <c r="D71" s="23">
         <v>0.25</v>
@@ -12544,10 +12547,10 @@
     </row>
     <row r="101" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A101" s="22" t="s">
+        <v>387</v>
+      </c>
+      <c r="B101" s="22" t="s">
         <v>388</v>
-      </c>
-      <c r="B101" s="22" t="s">
-        <v>389</v>
       </c>
       <c r="C101" s="22" t="s">
         <v>44</v>
@@ -14054,10 +14057,10 @@
     </row>
     <row r="115" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A115" s="22" t="s">
+        <v>391</v>
+      </c>
+      <c r="B115" s="22" t="s">
         <v>392</v>
-      </c>
-      <c r="B115" s="22" t="s">
-        <v>393</v>
       </c>
       <c r="C115" s="22" t="s">
         <v>47</v>
@@ -14354,11 +14357,11 @@
         <v>50180</v>
       </c>
       <c r="AA117" s="24">
-        <v>0</v>
+        <v>27120</v>
       </c>
       <c r="AB117" s="20">
         <f>Z117-AA117</f>
-        <v>50180</v>
+        <v>23060</v>
       </c>
       <c r="AC117" s="24" t="str">
         <f>IF(AND($T117=6000, ($T117+$W117-$AB117)&gt;=6000),T117,"")</f>
@@ -14462,11 +14465,11 @@
         <v>72310</v>
       </c>
       <c r="AA118" s="24">
-        <v>0</v>
+        <v>27120</v>
       </c>
       <c r="AB118" s="20">
         <f>Z118-AA118</f>
-        <v>72310</v>
+        <v>45190</v>
       </c>
       <c r="AC118" s="24" t="str">
         <f>IF(AND($T118=6000, ($T118+$W118-$AB118)&gt;=6000),T118,"")</f>
@@ -16620,11 +16623,11 @@
         <v>46880</v>
       </c>
       <c r="AA138" s="24">
-        <v>30000</v>
+        <v>46880</v>
       </c>
       <c r="AB138" s="20">
         <f>Z138-AA138</f>
-        <v>16880</v>
+        <v>0</v>
       </c>
       <c r="AC138" s="24" t="str">
         <f>IF(AND($T138=6000, ($T138+$W138-$AB138)&gt;=6000),T138,"")</f>
@@ -16722,11 +16725,11 @@
       </c>
       <c r="AA139" s="28">
         <f>SUM(AA2:AA138)</f>
-        <v>3390735</v>
+        <v>3461855</v>
       </c>
       <c r="AB139" s="28">
         <f>SUM(AB2:AB138)</f>
-        <v>5479325</v>
+        <v>5408205</v>
       </c>
       <c r="AC139" s="28">
         <f>SUM(AC2:AC138)</f>
@@ -24213,7 +24216,7 @@
     <sortCondition ref="A2:A139"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="AC1:AF10 E139:AF139 AB140:AB996 AB1:AB138">
+  <conditionalFormatting sqref="AC1:AF10 AB1:AB138 E139:AF139 AB140:AB996">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
@@ -24267,7 +24270,7 @@
       </c>
       <c r="F1" s="36">
         <f>SUMIF(E1:E1000, "&lt;&gt;", D1:D1000)</f>
-        <v>3390735</v>
+        <v>3461855</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
@@ -25067,7 +25070,7 @@
         <v>50000</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
@@ -25097,13 +25100,13 @@
         <v>250</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D30" s="9">
         <v>30000</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
@@ -25745,13 +25748,13 @@
         <v>250</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D48" s="9">
         <v>100000</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
@@ -26033,13 +26036,13 @@
         <v>250</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D56" s="9">
         <v>22000</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="F56" s="7"/>
       <c r="G56" s="7"/>
@@ -26321,13 +26324,13 @@
         <v>250</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D64" s="9">
         <v>124270</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
@@ -26399,7 +26402,7 @@
         <v>80000</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F66" s="7"/>
       <c r="G66" s="7"/>
@@ -26423,19 +26426,19 @@
     </row>
     <row r="67" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="B67" s="7" t="s">
         <v>270</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>272</v>
+        <v>404</v>
       </c>
       <c r="D67" s="9">
-        <v>50000</v>
+        <v>54240</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>273</v>
+        <v>405</v>
       </c>
       <c r="F67" s="7"/>
       <c r="G67" s="7"/>
@@ -26459,19 +26462,19 @@
     </row>
     <row r="68" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>315</v>
+        <v>272</v>
       </c>
       <c r="D68" s="9">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>329</v>
+        <v>273</v>
       </c>
       <c r="F68" s="7"/>
       <c r="G68" s="7"/>
@@ -26495,19 +26498,19 @@
     </row>
     <row r="69" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
-        <v>46285</v>
+        <v>46280</v>
       </c>
       <c r="B69" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>371</v>
+        <v>315</v>
       </c>
       <c r="D69" s="9">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>383</v>
+        <v>329</v>
       </c>
       <c r="F69" s="7"/>
       <c r="G69" s="7"/>
@@ -26531,19 +26534,19 @@
     </row>
     <row r="70" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="8">
-        <v>46277</v>
+        <v>46285</v>
       </c>
       <c r="B70" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>294</v>
+        <v>371</v>
       </c>
       <c r="D70" s="9">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>297</v>
+        <v>383</v>
       </c>
       <c r="F70" s="7"/>
       <c r="G70" s="7"/>
@@ -26567,19 +26570,19 @@
     </row>
     <row r="71" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
-        <v>46280</v>
+        <v>46277</v>
       </c>
       <c r="B71" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>317</v>
+        <v>294</v>
       </c>
       <c r="D71" s="9">
-        <v>44140</v>
+        <v>10000</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>348</v>
+        <v>297</v>
       </c>
       <c r="F71" s="7"/>
       <c r="G71" s="7"/>
@@ -26603,19 +26606,19 @@
     </row>
     <row r="72" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="B72" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>263</v>
+        <v>317</v>
       </c>
       <c r="D72" s="9">
-        <v>50000</v>
+        <v>44140</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>264</v>
+        <v>348</v>
       </c>
       <c r="F72" s="7"/>
       <c r="G72" s="7"/>
@@ -26639,19 +26642,19 @@
     </row>
     <row r="73" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
-        <v>46281</v>
+        <v>46266</v>
       </c>
       <c r="B73" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>345</v>
+        <v>263</v>
       </c>
       <c r="D73" s="9">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>346</v>
+        <v>264</v>
       </c>
       <c r="F73" s="7"/>
       <c r="G73" s="7"/>
@@ -26675,7 +26678,7 @@
     </row>
     <row r="74" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
-        <v>46286</v>
+        <v>46281</v>
       </c>
       <c r="B74" s="7" t="s">
         <v>250</v>
@@ -26684,7 +26687,7 @@
         <v>345</v>
       </c>
       <c r="D74" s="9">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>346</v>
@@ -26711,18 +26714,20 @@
     </row>
     <row r="75" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
-        <v>46279</v>
+        <v>46286</v>
       </c>
       <c r="B75" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>309</v>
+        <v>345</v>
       </c>
       <c r="D75" s="9">
-        <v>36050</v>
-      </c>
-      <c r="E75" s="7"/>
+        <v>10000</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>346</v>
+      </c>
       <c r="F75" s="7"/>
       <c r="G75" s="7"/>
       <c r="H75" s="7"/>
@@ -26745,18 +26750,20 @@
     </row>
     <row r="76" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
-        <v>46279</v>
+        <v>46290</v>
       </c>
       <c r="B76" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>310</v>
+        <v>345</v>
       </c>
       <c r="D76" s="9">
-        <v>100000</v>
-      </c>
-      <c r="E76" s="7"/>
+        <v>16880</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>346</v>
+      </c>
       <c r="F76" s="7"/>
       <c r="G76" s="7"/>
       <c r="H76" s="7"/>
@@ -26782,13 +26789,13 @@
         <v>46279</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D77" s="9">
-        <v>20180</v>
+        <v>36050</v>
       </c>
       <c r="E77" s="7"/>
       <c r="F77" s="7"/>
@@ -26813,18 +26820,18 @@
     </row>
     <row r="78" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="8">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B78" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C78" s="11" t="s">
-        <v>316</v>
-      </c>
-      <c r="D78" s="12">
-        <v>10000</v>
-      </c>
-      <c r="E78" s="11"/>
+      <c r="C78" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="D78" s="9">
+        <v>100000</v>
+      </c>
+      <c r="E78" s="7"/>
       <c r="F78" s="7"/>
       <c r="G78" s="7"/>
       <c r="H78" s="7"/>
@@ -26847,16 +26854,16 @@
     </row>
     <row r="79" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="D79" s="9">
-        <v>10000</v>
+        <v>20180</v>
       </c>
       <c r="E79" s="7"/>
       <c r="F79" s="7"/>
@@ -26881,18 +26888,18 @@
     </row>
     <row r="80" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="B80" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="C80" s="7" t="s">
-        <v>364</v>
-      </c>
-      <c r="D80" s="9">
-        <v>40000</v>
-      </c>
-      <c r="E80" s="7"/>
+      <c r="C80" s="11" t="s">
+        <v>316</v>
+      </c>
+      <c r="D80" s="12">
+        <v>10000</v>
+      </c>
+      <c r="E80" s="11"/>
       <c r="F80" s="7"/>
       <c r="G80" s="7"/>
       <c r="H80" s="7"/>
@@ -26915,16 +26922,16 @@
     </row>
     <row r="81" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
-        <v>46286</v>
+        <v>46281</v>
       </c>
       <c r="B81" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>372</v>
+        <v>316</v>
       </c>
       <c r="D81" s="9">
-        <v>90000</v>
+        <v>10000</v>
       </c>
       <c r="E81" s="7"/>
       <c r="F81" s="7"/>
@@ -26949,13 +26956,13 @@
     </row>
     <row r="82" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
-        <v>46288</v>
+        <v>46282</v>
       </c>
       <c r="B82" s="7" t="s">
         <v>250</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>396</v>
+        <v>364</v>
       </c>
       <c r="D82" s="9">
         <v>40000</v>
@@ -26982,9 +26989,18 @@
       <c r="X82" s="7"/>
     </row>
     <row r="83" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="7"/>
-      <c r="C83" s="7"/>
-      <c r="D83" s="9"/>
+      <c r="A83" s="8">
+        <v>46286</v>
+      </c>
+      <c r="B83" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="D83" s="9">
+        <v>90000</v>
+      </c>
       <c r="E83" s="7"/>
       <c r="F83" s="7"/>
       <c r="G83" s="7"/>
@@ -27007,9 +27023,18 @@
       <c r="X83" s="7"/>
     </row>
     <row r="84" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="7"/>
-      <c r="C84" s="7"/>
-      <c r="D84" s="9"/>
+      <c r="A84" s="8">
+        <v>46288</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="D84" s="9">
+        <v>40000</v>
+      </c>
       <c r="E84" s="7"/>
       <c r="F84" s="7"/>
       <c r="G84" s="7"/>
@@ -39656,8 +39681,8 @@
       <c r="X589" s="7"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F82">
-    <sortCondition ref="E2:E82"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F84">
+    <sortCondition ref="E2:E84"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Correct student fee balances and totals
Updated the fee ledger data in the Excel files and student term JSON so payment totals, balances, and outstanding amounts match the actual records. This fixes incorrect zero-balance and overpaid entries, corrects negative balances, and keeps the parent-code data aligned with the revised student fee records.
</commit_message>
<xml_diff>
--- a/2026 - 2027 FEE.xlsx
+++ b/2026 - 2027 FEE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\KBI\ACCOUNTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D799A21-B48E-409D-889E-46CC2C55949A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA151B7-FEDC-401E-BF98-A24C0BDECEB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="781" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1ST TERM ACCOUNT" sheetId="14" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="938" uniqueCount="462">
   <si>
     <t>LAST NAME</t>
   </si>
@@ -1403,6 +1403,27 @@
   <si>
     <t>AWODOLA JOSHUA AYOMIDE</t>
   </si>
+  <si>
+    <t>For Orinayo and Imoleayo Oyetunji</t>
+  </si>
+  <si>
+    <t>NIP:AKINYEMI AKINPELU TIMOTHY-</t>
+  </si>
+  <si>
+    <t>AYOBAMI KASALI - Abdulazeez Abdullah Balance</t>
+  </si>
+  <si>
+    <t>AKINYEMI DANIEL</t>
+  </si>
+  <si>
+    <t>OYETUNJI FAMILY</t>
+  </si>
+  <si>
+    <t>NIP:SAHEED ADEKUNLE ADEBUNMI</t>
+  </si>
+  <si>
+    <t>ADEBUNMI FAMILY</t>
+  </si>
 </sst>
 </file>
 
@@ -2116,15 +2137,15 @@
         <v>51180</v>
       </c>
       <c r="AA2" s="24">
-        <v>30000</v>
+        <v>51180</v>
       </c>
       <c r="AB2" s="20">
         <f t="shared" ref="AB2:AB33" si="6">Z2-AA2</f>
-        <v>21180</v>
-      </c>
-      <c r="AC2" s="24" t="str">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="24">
         <f t="shared" ref="AC2:AC33" si="7">IF(AND($T2=6000, ($T2+$W2-$AB2)&gt;=6000),T2,"")</f>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="AD2" s="24" t="str">
         <f t="shared" ref="AD2:AD33" si="8">IF(AND($T2=8000, ($T2+$W2-$AB2)&gt;=8000),T2,"")</f>
@@ -3415,11 +3436,11 @@
         <v>52660</v>
       </c>
       <c r="AA14" s="24">
-        <v>0</v>
+        <v>52660</v>
       </c>
       <c r="AB14" s="20">
         <f t="shared" si="6"/>
-        <v>52660</v>
+        <v>0</v>
       </c>
       <c r="AC14" s="24" t="str">
         <f t="shared" si="7"/>
@@ -3523,11 +3544,11 @@
         <v>60510</v>
       </c>
       <c r="AA15" s="24">
-        <v>0</v>
+        <v>61090</v>
       </c>
       <c r="AB15" s="20">
         <f t="shared" si="6"/>
-        <v>60510</v>
+        <v>-580</v>
       </c>
       <c r="AC15" s="24" t="str">
         <f t="shared" si="7"/>
@@ -6223,15 +6244,15 @@
         <v>56930</v>
       </c>
       <c r="AA40" s="24">
-        <v>0</v>
+        <v>56930</v>
       </c>
       <c r="AB40" s="20">
         <f t="shared" si="16"/>
-        <v>56930</v>
-      </c>
-      <c r="AC40" s="24" t="str">
+        <v>0</v>
+      </c>
+      <c r="AC40" s="24">
         <f t="shared" si="17"/>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="AD40" s="24" t="str">
         <f t="shared" si="18"/>
@@ -7522,15 +7543,15 @@
         <v>82800</v>
       </c>
       <c r="AA52" s="24">
-        <v>82350</v>
+        <v>82800</v>
       </c>
       <c r="AB52" s="20">
         <f t="shared" si="16"/>
-        <v>450</v>
-      </c>
-      <c r="AC52" s="24" t="str">
+        <v>0</v>
+      </c>
+      <c r="AC52" s="24">
         <f t="shared" si="17"/>
-        <v/>
+        <v>6000</v>
       </c>
       <c r="AD52" s="24" t="str">
         <f t="shared" si="18"/>
@@ -14835,11 +14856,11 @@
         <v>24550</v>
       </c>
       <c r="AA120" s="24">
-        <v>0</v>
+        <v>24550</v>
       </c>
       <c r="AB120" s="20">
         <f t="shared" si="39"/>
-        <v>24550</v>
+        <v>0</v>
       </c>
       <c r="AC120" s="24" t="str">
         <f t="shared" si="30"/>
@@ -14943,11 +14964,11 @@
         <v>81160</v>
       </c>
       <c r="AA121" s="24">
-        <v>0</v>
+        <v>25450</v>
       </c>
       <c r="AB121" s="20">
         <f t="shared" si="39"/>
-        <v>81160</v>
+        <v>55710</v>
       </c>
       <c r="AC121" s="24" t="str">
         <f t="shared" si="30"/>
@@ -15910,14 +15931,14 @@
         <v>0</v>
       </c>
       <c r="Z130" s="24">
-        <f t="shared" ref="Z130:Z161" si="45">SUM(J130:Y130)</f>
+        <f t="shared" ref="Z130:Z136" si="45">SUM(J130:Y130)</f>
         <v>75310</v>
       </c>
       <c r="AA130" s="24">
         <v>20000</v>
       </c>
       <c r="AB130" s="20">
-        <f t="shared" ref="AB130:AB161" si="46">Z130-AA130</f>
+        <f t="shared" ref="AB130:AB136" si="46">Z130-AA130</f>
         <v>55310</v>
       </c>
       <c r="AC130" s="24" t="str">
@@ -16666,15 +16687,15 @@
       </c>
       <c r="AA137" s="28">
         <f t="shared" si="47"/>
-        <v>5021955</v>
+        <v>5264265</v>
       </c>
       <c r="AB137" s="28">
         <f t="shared" si="47"/>
-        <v>3639155</v>
+        <v>3396845</v>
       </c>
       <c r="AC137" s="28">
         <f t="shared" si="47"/>
-        <v>60000</v>
+        <v>78000</v>
       </c>
       <c r="AD137" s="28">
         <f t="shared" si="47"/>
@@ -24211,7 +24232,7 @@
       </c>
       <c r="F1" s="36">
         <f>SUMIF(E1:E1000, "&lt;&gt;", D1:D1000)</f>
-        <v>5021955</v>
+        <v>5264265</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
@@ -24234,209 +24255,209 @@
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
-        <v>46238</v>
+        <v>46278</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>242</v>
+        <v>293</v>
       </c>
       <c r="D2" s="9">
-        <v>48000</v>
+        <v>60000</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>244</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
-        <v>46255</v>
+        <v>46306</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>246</v>
+        <v>457</v>
       </c>
       <c r="D3" s="9">
-        <v>43000</v>
+        <v>21180</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>247</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
-        <v>46262</v>
+        <v>46300</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>246</v>
+        <v>440</v>
       </c>
       <c r="D4" s="9">
-        <v>33000</v>
+        <v>40000</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>247</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
-        <v>46262</v>
+        <v>46277</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>246</v>
+        <v>288</v>
       </c>
       <c r="D5" s="9">
-        <v>615</v>
+        <v>30000</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>247</v>
+        <v>289</v>
       </c>
       <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
-        <v>46263</v>
+        <v>46265</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="D6" s="9">
-        <v>18000</v>
+        <v>60000</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
-        <v>46264</v>
+        <v>46280</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="D7" s="9">
-        <v>51930</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>250</v>
+      <c r="C7" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="D7" s="12">
+        <v>40000</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
-        <v>46265</v>
+        <v>46282</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>252</v>
+        <v>313</v>
       </c>
       <c r="D8" s="9">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>254</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
-        <v>46265</v>
+        <v>46286</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>253</v>
+        <v>313</v>
       </c>
       <c r="D9" s="9">
-        <v>50430</v>
+        <v>29000</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>255</v>
+        <v>359</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
-        <v>46266</v>
+        <v>46286</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>256</v>
+        <v>366</v>
       </c>
       <c r="D10" s="9">
         <v>50000</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>257</v>
+        <v>373</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
-        <v>46268</v>
+        <v>46299</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>258</v>
+        <v>366</v>
       </c>
       <c r="D11" s="9">
-        <v>42140</v>
+        <v>20000</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>259</v>
+        <v>373</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
-        <v>46270</v>
+        <v>46268</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D12" s="9">
-        <v>79020</v>
+        <v>42140</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
-        <v>46270</v>
+        <v>46280</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>264</v>
+        <v>330</v>
       </c>
       <c r="D13" s="9">
-        <v>42350</v>
+        <v>80000</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="F13" s="7"/>
+        <v>331</v>
+      </c>
+      <c r="F13" s="11"/>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
@@ -24458,19 +24479,19 @@
     </row>
     <row r="14" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
-        <v>46270</v>
+        <v>46280</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>265</v>
+        <v>311</v>
       </c>
       <c r="D14" s="9">
-        <v>50000</v>
+        <v>120210</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>266</v>
+        <v>329</v>
       </c>
       <c r="F14" s="7"/>
       <c r="G14" s="7"/>
@@ -24494,19 +24515,19 @@
     </row>
     <row r="15" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
-        <v>46271</v>
+        <v>46255</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="D15" s="9">
-        <v>60000</v>
+        <v>43000</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
@@ -24529,20 +24550,20 @@
       <c r="X15" s="7"/>
     </row>
     <row r="16" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10">
-        <v>46271</v>
-      </c>
-      <c r="B16" s="11" t="s">
+      <c r="A16" s="8">
+        <v>46262</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="C16" s="11" t="s">
-        <v>269</v>
-      </c>
-      <c r="D16" s="12">
-        <v>20000</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>276</v>
+      <c r="C16" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="D16" s="9">
+        <v>33000</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>247</v>
       </c>
       <c r="F16" s="7"/>
       <c r="G16" s="7"/>
@@ -24566,19 +24587,19 @@
     </row>
     <row r="17" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
-        <v>46273</v>
+        <v>46262</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>270</v>
+        <v>246</v>
       </c>
       <c r="D17" s="9">
-        <v>33000</v>
+        <v>615</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>275</v>
+        <v>247</v>
       </c>
       <c r="F17" s="7"/>
       <c r="G17" s="7"/>
@@ -24602,19 +24623,19 @@
     </row>
     <row r="18" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
-        <v>46273</v>
+        <v>46263</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>271</v>
+        <v>246</v>
       </c>
       <c r="D18" s="9">
-        <v>6840</v>
+        <v>18000</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>275</v>
+        <v>247</v>
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="7"/>
@@ -24638,19 +24659,19 @@
     </row>
     <row r="19" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
-        <v>46273</v>
+        <v>46278</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>272</v>
+        <v>298</v>
       </c>
       <c r="D19" s="9">
-        <v>200000</v>
+        <v>30000</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>274</v>
+        <v>247</v>
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="7"/>
@@ -24674,19 +24695,19 @@
     </row>
     <row r="20" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
-        <v>46275</v>
+        <v>46279</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>279</v>
+        <v>298</v>
       </c>
       <c r="D20" s="9">
-        <v>24700</v>
+        <v>8000</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>280</v>
+        <v>247</v>
       </c>
       <c r="F20" s="7"/>
       <c r="G20" s="7"/>
@@ -24709,22 +24730,22 @@
       <c r="X20" s="7"/>
     </row>
     <row r="21" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10">
-        <v>46275</v>
-      </c>
-      <c r="B21" s="11" t="s">
+      <c r="A21" s="8">
+        <v>46280</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="C21" s="11" t="s">
-        <v>278</v>
-      </c>
-      <c r="D21" s="12">
-        <v>33140</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>277</v>
-      </c>
-      <c r="F21" s="7"/>
+      <c r="C21" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="D21" s="9">
+        <v>20000</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="F21" s="11"/>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
@@ -24746,19 +24767,19 @@
     </row>
     <row r="22" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
-        <v>46276</v>
+        <v>46295</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
       <c r="D22" s="9">
-        <v>28000</v>
+        <v>48000</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>291</v>
+        <v>247</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
@@ -24782,19 +24803,19 @@
     </row>
     <row r="23" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
-        <v>46277</v>
+        <v>46300</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>288</v>
+        <v>439</v>
       </c>
       <c r="D23" s="9">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>289</v>
+        <v>451</v>
       </c>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
@@ -24818,19 +24839,19 @@
     </row>
     <row r="24" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="D24" s="9">
-        <v>95000</v>
+        <v>62230</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
@@ -24854,19 +24875,19 @@
     </row>
     <row r="25" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
-        <v>46277</v>
+        <v>46271</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>287</v>
+        <v>260</v>
       </c>
       <c r="D25" s="9">
-        <v>10000</v>
+        <v>60000</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>290</v>
+        <v>261</v>
       </c>
       <c r="F25" s="7"/>
       <c r="G25" s="7"/>
@@ -24890,19 +24911,19 @@
     </row>
     <row r="26" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>293</v>
+        <v>369</v>
       </c>
       <c r="D26" s="9">
-        <v>60000</v>
+        <v>27000</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>297</v>
+        <v>372</v>
       </c>
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
@@ -24926,19 +24947,19 @@
     </row>
     <row r="27" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
-        <v>46278</v>
+        <v>46286</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>298</v>
+        <v>370</v>
       </c>
       <c r="D27" s="9">
-        <v>30000</v>
+        <v>16140</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>247</v>
+        <v>372</v>
       </c>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
@@ -24962,19 +24983,19 @@
     </row>
     <row r="28" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
-        <v>46278</v>
+        <v>46280</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>294</v>
+        <v>314</v>
       </c>
       <c r="D28" s="9">
-        <v>62230</v>
+        <v>40000</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>296</v>
+        <v>320</v>
       </c>
       <c r="F28" s="7"/>
       <c r="G28" s="7"/>
@@ -25034,19 +25055,19 @@
     </row>
     <row r="30" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
-        <v>46278</v>
+        <v>46280</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>292</v>
+        <v>312</v>
       </c>
       <c r="D30" s="9">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>295</v>
+        <v>326</v>
       </c>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
@@ -25070,19 +25091,19 @@
     </row>
     <row r="31" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
-        <v>46278</v>
+        <v>46265</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>269</v>
+        <v>253</v>
       </c>
       <c r="D31" s="9">
-        <v>9640</v>
+        <v>50430</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>276</v>
+        <v>255</v>
       </c>
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
@@ -25106,19 +25127,19 @@
     </row>
     <row r="32" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
-        <v>46279</v>
+        <v>46301</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>298</v>
+        <v>447</v>
       </c>
       <c r="D32" s="9">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
@@ -25142,19 +25163,19 @@
     </row>
     <row r="33" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
-        <v>46279</v>
+        <v>46297</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>303</v>
+        <v>426</v>
       </c>
       <c r="D33" s="9">
-        <v>100000</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>411</v>
+        <v>70000</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>434</v>
       </c>
       <c r="F33" s="7"/>
       <c r="G33" s="7"/>
@@ -25178,19 +25199,19 @@
     </row>
     <row r="34" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
-        <v>46279</v>
+        <v>46276</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>305</v>
+        <v>284</v>
       </c>
       <c r="D34" s="9">
-        <v>25000</v>
+        <v>28000</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
@@ -25214,19 +25235,19 @@
     </row>
     <row r="35" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>301</v>
+        <v>284</v>
       </c>
       <c r="D35" s="9">
-        <v>116000</v>
+        <v>15140</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>356</v>
+        <v>291</v>
       </c>
       <c r="F35" s="7"/>
       <c r="G35" s="7"/>
@@ -25250,19 +25271,19 @@
     </row>
     <row r="36" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
-        <v>46279</v>
+        <v>46306</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>279</v>
+        <v>456</v>
       </c>
       <c r="D36" s="9">
-        <v>20000</v>
+        <v>56930</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>280</v>
+        <v>458</v>
       </c>
       <c r="F36" s="7"/>
       <c r="G36" s="7"/>
@@ -25286,19 +25307,19 @@
     </row>
     <row r="37" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>302</v>
+        <v>358</v>
       </c>
       <c r="D37" s="9">
-        <v>36050</v>
+        <v>50000</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>410</v>
+        <v>394</v>
       </c>
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
@@ -25322,18 +25343,20 @@
     </row>
     <row r="38" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
-        <v>46279</v>
+        <v>46301</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>304</v>
+        <v>443</v>
       </c>
       <c r="D38" s="9">
-        <v>20180</v>
-      </c>
-      <c r="E38" s="7"/>
+        <v>20000</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>449</v>
+      </c>
       <c r="F38" s="7"/>
       <c r="G38" s="7"/>
       <c r="H38" s="7"/>
@@ -25356,19 +25379,19 @@
     </row>
     <row r="39" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
-        <v>46280</v>
+        <v>46287</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="C39" s="11" t="s">
-        <v>313</v>
-      </c>
-      <c r="D39" s="12">
-        <v>40000</v>
-      </c>
-      <c r="E39" s="11" t="s">
-        <v>359</v>
+      <c r="C39" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="D39" s="9">
+        <v>30000</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>392</v>
       </c>
       <c r="F39" s="7"/>
       <c r="G39" s="7"/>
@@ -25392,21 +25415,21 @@
     </row>
     <row r="40" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
-        <v>46280</v>
+        <v>46300</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>330</v>
+        <v>429</v>
       </c>
       <c r="D40" s="9">
-        <v>80000</v>
+        <v>25000</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="F40" s="11"/>
+        <v>433</v>
+      </c>
+      <c r="F40" s="7"/>
       <c r="G40" s="7"/>
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
@@ -25428,19 +25451,19 @@
     </row>
     <row r="41" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
-        <v>46280</v>
+        <v>46302</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>311</v>
+        <v>452</v>
       </c>
       <c r="D41" s="9">
-        <v>120210</v>
+        <v>30000</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>329</v>
+        <v>454</v>
       </c>
       <c r="F41" s="7"/>
       <c r="G41" s="7"/>
@@ -25464,21 +25487,21 @@
     </row>
     <row r="42" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
-        <v>46280</v>
+        <v>46278</v>
       </c>
       <c r="B42" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="D42" s="9">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="F42" s="11"/>
+        <v>295</v>
+      </c>
+      <c r="F42" s="7"/>
       <c r="G42" s="7"/>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
@@ -25500,19 +25523,19 @@
     </row>
     <row r="43" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
-        <v>46280</v>
+        <v>46301</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>314</v>
+        <v>445</v>
       </c>
       <c r="D43" s="9">
-        <v>40000</v>
+        <v>30000</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>320</v>
+        <v>448</v>
       </c>
       <c r="F43" s="7"/>
       <c r="G43" s="7"/>
@@ -25536,19 +25559,19 @@
     </row>
     <row r="44" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>312</v>
+        <v>262</v>
       </c>
       <c r="D44" s="9">
-        <v>60000</v>
+        <v>79020</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>326</v>
+        <v>268</v>
       </c>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
@@ -25572,19 +25595,19 @@
     </row>
     <row r="45" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
-        <v>46280</v>
+        <v>46238</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>284</v>
+        <v>242</v>
       </c>
       <c r="D45" s="9">
-        <v>15140</v>
+        <v>48000</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>291</v>
+        <v>244</v>
       </c>
       <c r="F45" s="7"/>
       <c r="G45" s="7"/>
@@ -25608,19 +25631,19 @@
     </row>
     <row r="46" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
-        <v>46280</v>
+        <v>46282</v>
       </c>
       <c r="B46" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="C46" s="11" t="s">
-        <v>316</v>
-      </c>
-      <c r="D46" s="12">
-        <v>40000</v>
-      </c>
-      <c r="E46" s="11" t="s">
-        <v>321</v>
+      <c r="C46" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="D46" s="9">
+        <v>35180</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>244</v>
       </c>
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
@@ -25644,19 +25667,19 @@
     </row>
     <row r="47" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>335</v>
+        <v>264</v>
       </c>
       <c r="D47" s="9">
-        <v>50000</v>
+        <v>42350</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>336</v>
+        <v>267</v>
       </c>
       <c r="F47" s="7"/>
       <c r="G47" s="7"/>
@@ -25680,19 +25703,19 @@
     </row>
     <row r="48" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
-        <v>46280</v>
+        <v>46282</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>307</v>
+        <v>264</v>
       </c>
       <c r="D48" s="9">
-        <v>30000</v>
+        <v>40000</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>362</v>
+        <v>267</v>
       </c>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
@@ -25716,19 +25739,19 @@
     </row>
     <row r="49" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
-        <v>46280</v>
+        <v>46306</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>309</v>
-      </c>
-      <c r="D49" s="12">
-        <v>10000</v>
-      </c>
-      <c r="E49" s="11" t="s">
-        <v>412</v>
+        <v>263</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="D49" s="9">
+        <v>450</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>267</v>
       </c>
       <c r="F49" s="7"/>
       <c r="G49" s="11"/>
@@ -25752,21 +25775,21 @@
     </row>
     <row r="50" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="B50" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>332</v>
+        <v>303</v>
       </c>
       <c r="D50" s="9">
-        <v>65160</v>
+        <v>100000</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="F50" s="11"/>
+        <v>411</v>
+      </c>
+      <c r="F50" s="7"/>
       <c r="G50" s="11"/>
       <c r="H50" s="11"/>
       <c r="I50" s="11"/>
@@ -25793,16 +25816,16 @@
       <c r="B51" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="C51" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="D51" s="9">
-        <v>35890</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>334</v>
-      </c>
-      <c r="F51" s="11"/>
+      <c r="C51" s="11" t="s">
+        <v>316</v>
+      </c>
+      <c r="D51" s="12">
+        <v>40000</v>
+      </c>
+      <c r="E51" s="11" t="s">
+        <v>321</v>
+      </c>
+      <c r="F51" s="7"/>
       <c r="G51" s="11"/>
       <c r="H51" s="11"/>
       <c r="I51" s="11"/>
@@ -25824,19 +25847,19 @@
     </row>
     <row r="52" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
-        <v>46280</v>
+        <v>46289</v>
       </c>
       <c r="B52" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>337</v>
+        <v>316</v>
       </c>
       <c r="D52" s="9">
-        <v>50000</v>
+        <v>88000</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>340</v>
+        <v>321</v>
       </c>
       <c r="F52" s="7"/>
       <c r="G52" s="11"/>
@@ -25860,19 +25883,19 @@
     </row>
     <row r="53" spans="1:24" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
-        <v>46280</v>
+        <v>46273</v>
       </c>
       <c r="B53" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>315</v>
+        <v>270</v>
       </c>
       <c r="D53" s="9">
-        <v>27900</v>
+        <v>33000</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>317</v>
+        <v>275</v>
       </c>
       <c r="F53" s="7"/>
       <c r="G53" s="11"/>
@@ -25896,19 +25919,19 @@
     </row>
     <row r="54" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
-        <v>46280</v>
+        <v>46273</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>308</v>
+        <v>271</v>
       </c>
       <c r="D54" s="9">
-        <v>100000</v>
+        <v>6840</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>322</v>
+        <v>275</v>
       </c>
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
@@ -25932,21 +25955,21 @@
     </row>
     <row r="55" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>310</v>
+        <v>271</v>
       </c>
       <c r="D55" s="9">
-        <v>44140</v>
+        <v>5300</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>341</v>
-      </c>
-      <c r="F55" s="7"/>
+        <v>275</v>
+      </c>
+      <c r="F55" s="11"/>
       <c r="G55" s="7"/>
       <c r="H55" s="7"/>
       <c r="I55" s="7"/>
@@ -25982,7 +26005,7 @@
       <c r="E56" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="F56" s="11"/>
+      <c r="F56" s="7"/>
       <c r="G56" s="7"/>
       <c r="H56" s="7"/>
       <c r="I56" s="7"/>
@@ -26004,19 +26027,19 @@
     </row>
     <row r="57" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
-        <v>46281</v>
+        <v>46273</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>263</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D57" s="9">
-        <v>5300</v>
+        <v>200000</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
@@ -26040,19 +26063,19 @@
     </row>
     <row r="58" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8">
-        <v>46281</v>
+        <v>46286</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>309</v>
+        <v>371</v>
       </c>
       <c r="D58" s="9">
-        <v>10000</v>
+        <v>56930</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>412</v>
+        <v>377</v>
       </c>
       <c r="F58" s="7"/>
       <c r="G58" s="7"/>
@@ -26076,19 +26099,19 @@
     </row>
     <row r="59" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8">
-        <v>46281</v>
+        <v>46300</v>
       </c>
       <c r="B59" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>338</v>
+        <v>430</v>
       </c>
       <c r="D59" s="9">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>339</v>
+        <v>432</v>
       </c>
       <c r="F59" s="7"/>
       <c r="G59" s="7"/>
@@ -26112,19 +26135,19 @@
     </row>
     <row r="60" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8">
-        <v>46282</v>
+        <v>46297</v>
       </c>
       <c r="B60" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>313</v>
+        <v>427</v>
       </c>
       <c r="D60" s="9">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>359</v>
+        <v>435</v>
       </c>
       <c r="F60" s="7"/>
       <c r="G60" s="7"/>
@@ -26148,19 +26171,19 @@
     </row>
     <row r="61" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8">
-        <v>46282</v>
+        <v>46264</v>
       </c>
       <c r="B61" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="D61" s="9">
-        <v>35180</v>
+        <v>51930</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="F61" s="7"/>
       <c r="G61" s="7"/>
@@ -26184,19 +26207,19 @@
     </row>
     <row r="62" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="8">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="B62" s="7" t="s">
         <v>263</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>264</v>
+        <v>305</v>
       </c>
       <c r="D62" s="9">
-        <v>40000</v>
+        <v>25000</v>
       </c>
       <c r="E62" s="7" t="s">
-        <v>267</v>
+        <v>306</v>
       </c>
       <c r="F62" s="7"/>
       <c r="G62" s="7"/>
@@ -26220,19 +26243,19 @@
     </row>
     <row r="63" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="8">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="B63" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>357</v>
+        <v>335</v>
       </c>
       <c r="D63" s="9">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="E63" s="7" t="s">
-        <v>425</v>
+        <v>336</v>
       </c>
       <c r="F63" s="7"/>
       <c r="G63" s="7"/>
@@ -26256,19 +26279,19 @@
     </row>
     <row r="64" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="8">
-        <v>46283</v>
+        <v>46288</v>
       </c>
       <c r="B64" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>358</v>
+        <v>388</v>
       </c>
       <c r="D64" s="9">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
@@ -26292,19 +26315,19 @@
     </row>
     <row r="65" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="8">
-        <v>46284</v>
+        <v>46280</v>
       </c>
       <c r="B65" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>363</v>
+        <v>307</v>
       </c>
       <c r="D65" s="9">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>375</v>
+        <v>362</v>
       </c>
       <c r="F65" s="7"/>
       <c r="G65" s="7"/>
@@ -26328,19 +26351,19 @@
     </row>
     <row r="66" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
-        <v>46285</v>
+        <v>46294</v>
       </c>
       <c r="B66" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>363</v>
+        <v>415</v>
       </c>
       <c r="D66" s="9">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>375</v>
+        <v>362</v>
       </c>
       <c r="F66" s="7"/>
       <c r="G66" s="7"/>
@@ -26364,19 +26387,19 @@
     </row>
     <row r="67" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
-        <v>46285</v>
+        <v>46280</v>
       </c>
       <c r="B67" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="C67" s="7" t="s">
-        <v>364</v>
-      </c>
-      <c r="D67" s="9">
-        <v>50000</v>
-      </c>
-      <c r="E67" s="7" t="s">
-        <v>376</v>
+      <c r="C67" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="D67" s="12">
+        <v>10000</v>
+      </c>
+      <c r="E67" s="11" t="s">
+        <v>412</v>
       </c>
       <c r="F67" s="7"/>
       <c r="G67" s="7"/>
@@ -26400,19 +26423,19 @@
     </row>
     <row r="68" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
-        <v>46286</v>
+        <v>46281</v>
       </c>
       <c r="B68" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D68" s="9">
-        <v>29000</v>
+        <v>10000</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>359</v>
+        <v>412</v>
       </c>
       <c r="F68" s="7"/>
       <c r="G68" s="7"/>
@@ -26436,19 +26459,19 @@
     </row>
     <row r="69" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="8">
-        <v>46286</v>
+        <v>46296</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>366</v>
+        <v>421</v>
       </c>
       <c r="D69" s="9">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>373</v>
+        <v>423</v>
       </c>
       <c r="F69" s="7"/>
       <c r="G69" s="7"/>
@@ -26471,20 +26494,20 @@
       <c r="X69" s="7"/>
     </row>
     <row r="70" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="8">
-        <v>46286</v>
-      </c>
-      <c r="B70" s="7" t="s">
+      <c r="A70" s="10">
+        <v>46271</v>
+      </c>
+      <c r="B70" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="C70" s="7" t="s">
-        <v>369</v>
-      </c>
-      <c r="D70" s="9">
-        <v>27000</v>
-      </c>
-      <c r="E70" s="7" t="s">
-        <v>372</v>
+      <c r="C70" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="D70" s="12">
+        <v>20000</v>
+      </c>
+      <c r="E70" s="11" t="s">
+        <v>276</v>
       </c>
       <c r="F70" s="7"/>
       <c r="G70" s="7"/>
@@ -26508,19 +26531,19 @@
     </row>
     <row r="71" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
-        <v>46286</v>
+        <v>46278</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>370</v>
+        <v>269</v>
       </c>
       <c r="D71" s="9">
-        <v>16140</v>
+        <v>9640</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>372</v>
+        <v>276</v>
       </c>
       <c r="F71" s="7"/>
       <c r="G71" s="7"/>
@@ -26544,19 +26567,19 @@
     </row>
     <row r="72" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
-        <v>46286</v>
+        <v>46292</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>371</v>
+        <v>402</v>
       </c>
       <c r="D72" s="9">
-        <v>56930</v>
+        <v>50000</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>377</v>
+        <v>406</v>
       </c>
       <c r="F72" s="7"/>
       <c r="G72" s="7"/>
@@ -26580,21 +26603,21 @@
     </row>
     <row r="73" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="B73" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>365</v>
+        <v>332</v>
       </c>
       <c r="D73" s="9">
-        <v>90000</v>
+        <v>65160</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>400</v>
-      </c>
-      <c r="F73" s="7"/>
+        <v>333</v>
+      </c>
+      <c r="F73" s="11"/>
       <c r="G73" s="7"/>
       <c r="H73" s="7"/>
       <c r="I73" s="7"/>
@@ -26616,21 +26639,21 @@
     </row>
     <row r="74" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="8">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="B74" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>368</v>
+        <v>332</v>
       </c>
       <c r="D74" s="9">
-        <v>50000</v>
+        <v>35890</v>
       </c>
       <c r="E74" s="7" t="s">
-        <v>374</v>
-      </c>
-      <c r="F74" s="7"/>
+        <v>334</v>
+      </c>
+      <c r="F74" s="11"/>
       <c r="G74" s="7"/>
       <c r="H74" s="7"/>
       <c r="I74" s="7"/>
@@ -26652,19 +26675,19 @@
     </row>
     <row r="75" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="8">
-        <v>46286</v>
+        <v>46299</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>367</v>
+        <v>304</v>
       </c>
       <c r="D75" s="9">
-        <v>80000</v>
+        <v>30000</v>
       </c>
       <c r="E75" s="7" t="s">
-        <v>393</v>
+        <v>431</v>
       </c>
       <c r="F75" s="7"/>
       <c r="G75" s="7"/>
@@ -26688,19 +26711,19 @@
     </row>
     <row r="76" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8">
-        <v>46286</v>
+        <v>46280</v>
       </c>
       <c r="B76" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D76" s="9">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="E76" s="7" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F76" s="7"/>
       <c r="G76" s="7"/>
@@ -26724,19 +26747,19 @@
     </row>
     <row r="77" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="8">
-        <v>46287</v>
+        <v>46279</v>
       </c>
       <c r="B77" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>424</v>
+        <v>301</v>
       </c>
       <c r="D77" s="9">
-        <v>30000</v>
+        <v>116000</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>392</v>
+        <v>356</v>
       </c>
       <c r="F77" s="7"/>
       <c r="G77" s="7"/>
@@ -26796,19 +26819,19 @@
     </row>
     <row r="79" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="8">
-        <v>46288</v>
+        <v>46294</v>
       </c>
       <c r="B79" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>388</v>
+        <v>414</v>
       </c>
       <c r="D79" s="9">
-        <v>100000</v>
+        <v>65000</v>
       </c>
       <c r="E79" s="7" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="F79" s="7"/>
       <c r="G79" s="7"/>
@@ -26832,19 +26855,19 @@
     </row>
     <row r="80" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="8">
-        <v>46288</v>
+        <v>46284</v>
       </c>
       <c r="B80" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>387</v>
+        <v>363</v>
       </c>
       <c r="D80" s="9">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="E80" s="7" t="s">
-        <v>413</v>
+        <v>375</v>
       </c>
       <c r="F80" s="7"/>
       <c r="G80" s="7"/>
@@ -26868,19 +26891,19 @@
     </row>
     <row r="81" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
-        <v>46288</v>
+        <v>46285</v>
       </c>
       <c r="B81" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>389</v>
+        <v>363</v>
       </c>
       <c r="D81" s="9">
-        <v>124270</v>
+        <v>50000</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>390</v>
+        <v>375</v>
       </c>
       <c r="F81" s="7"/>
       <c r="G81" s="7"/>
@@ -26904,19 +26927,19 @@
     </row>
     <row r="82" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8">
-        <v>46289</v>
+        <v>46300</v>
       </c>
       <c r="B82" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>316</v>
+        <v>428</v>
       </c>
       <c r="D82" s="9">
-        <v>88000</v>
+        <v>50000</v>
       </c>
       <c r="E82" s="7" t="s">
-        <v>321</v>
+        <v>436</v>
       </c>
       <c r="F82" s="7"/>
       <c r="G82" s="7"/>
@@ -26940,19 +26963,19 @@
     </row>
     <row r="83" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>396</v>
+        <v>365</v>
       </c>
       <c r="D83" s="9">
-        <v>54240</v>
+        <v>90000</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="F83" s="7"/>
       <c r="G83" s="7"/>
@@ -26976,19 +26999,19 @@
     </row>
     <row r="84" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="B84" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>338</v>
+        <v>368</v>
       </c>
       <c r="D84" s="9">
-        <v>16880</v>
+        <v>50000</v>
       </c>
       <c r="E84" s="7" t="s">
-        <v>339</v>
+        <v>374</v>
       </c>
       <c r="F84" s="7"/>
       <c r="G84" s="7"/>
@@ -27012,19 +27035,19 @@
     </row>
     <row r="85" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="8">
-        <v>46292</v>
+        <v>46282</v>
       </c>
       <c r="B85" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>402</v>
+        <v>357</v>
       </c>
       <c r="D85" s="9">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="E85" s="7" t="s">
-        <v>406</v>
+        <v>425</v>
       </c>
       <c r="F85" s="7"/>
       <c r="G85" s="7"/>
@@ -27048,19 +27071,19 @@
     </row>
     <row r="86" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="8">
-        <v>46292</v>
+        <v>46277</v>
       </c>
       <c r="B86" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>401</v>
+        <v>285</v>
       </c>
       <c r="D86" s="9">
-        <v>30000</v>
+        <v>95000</v>
       </c>
       <c r="E86" s="7" t="s">
-        <v>405</v>
+        <v>286</v>
       </c>
       <c r="F86" s="7"/>
       <c r="G86" s="7"/>
@@ -27084,19 +27107,19 @@
     </row>
     <row r="87" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="8">
-        <v>46293</v>
+        <v>46302</v>
       </c>
       <c r="B87" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>404</v>
+        <v>446</v>
       </c>
       <c r="D87" s="9">
-        <v>80000</v>
+        <v>49050</v>
       </c>
       <c r="E87" s="7" t="s">
-        <v>408</v>
+        <v>453</v>
       </c>
       <c r="F87" s="7"/>
       <c r="G87" s="7"/>
@@ -27126,13 +27149,13 @@
         <v>243</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>288</v>
+        <v>404</v>
       </c>
       <c r="D88" s="9">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="E88" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F88" s="7"/>
       <c r="G88" s="7"/>
@@ -27156,19 +27179,19 @@
     </row>
     <row r="89" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="8">
-        <v>46293</v>
+        <v>46280</v>
       </c>
       <c r="B89" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>403</v>
+        <v>315</v>
       </c>
       <c r="D89" s="9">
-        <v>50000</v>
+        <v>27900</v>
       </c>
       <c r="E89" s="7" t="s">
-        <v>409</v>
+        <v>317</v>
       </c>
       <c r="F89" s="7"/>
       <c r="G89" s="7"/>
@@ -27192,19 +27215,19 @@
     </row>
     <row r="90" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="8">
-        <v>46294</v>
+        <v>46288</v>
       </c>
       <c r="B90" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>415</v>
+        <v>387</v>
       </c>
       <c r="D90" s="9">
         <v>40000</v>
       </c>
       <c r="E90" s="7" t="s">
-        <v>362</v>
+        <v>413</v>
       </c>
       <c r="F90" s="7"/>
       <c r="G90" s="7"/>
@@ -27228,19 +27251,19 @@
     </row>
     <row r="91" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="8">
-        <v>46294</v>
+        <v>46301</v>
       </c>
       <c r="B91" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>414</v>
+        <v>444</v>
       </c>
       <c r="D91" s="9">
-        <v>65000</v>
+        <v>42000</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>395</v>
+        <v>413</v>
       </c>
       <c r="F91" s="7"/>
       <c r="G91" s="7"/>
@@ -27264,19 +27287,19 @@
     </row>
     <row r="92" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="8">
-        <v>46294</v>
+        <v>46275</v>
       </c>
       <c r="B92" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>417</v>
+        <v>279</v>
       </c>
       <c r="D92" s="9">
-        <v>140000</v>
+        <v>24700</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>419</v>
+        <v>280</v>
       </c>
       <c r="F92" s="7"/>
       <c r="G92" s="7"/>
@@ -27300,19 +27323,19 @@
     </row>
     <row r="93" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="8">
-        <v>46294</v>
+        <v>46279</v>
       </c>
       <c r="B93" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>416</v>
+        <v>279</v>
       </c>
       <c r="D93" s="9">
-        <v>40000</v>
+        <v>20000</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>418</v>
+        <v>280</v>
       </c>
       <c r="F93" s="7"/>
       <c r="G93" s="7"/>
@@ -27336,19 +27359,19 @@
     </row>
     <row r="94" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="8">
-        <v>46295</v>
+        <v>46294</v>
       </c>
       <c r="B94" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>298</v>
+        <v>417</v>
       </c>
       <c r="D94" s="9">
-        <v>48000</v>
+        <v>140000</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>247</v>
+        <v>419</v>
       </c>
       <c r="F94" s="7"/>
       <c r="G94" s="7"/>
@@ -27372,19 +27395,19 @@
     </row>
     <row r="95" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="8">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="B95" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>420</v>
+        <v>288</v>
       </c>
       <c r="D95" s="9">
-        <v>45000</v>
+        <v>30000</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
       <c r="F95" s="7"/>
       <c r="G95" s="7"/>
@@ -27408,19 +27431,19 @@
     </row>
     <row r="96" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="8">
-        <v>46296</v>
+        <v>46288</v>
       </c>
       <c r="B96" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>421</v>
+        <v>389</v>
       </c>
       <c r="D96" s="9">
-        <v>40000</v>
+        <v>124270</v>
       </c>
       <c r="E96" s="7" t="s">
-        <v>423</v>
+        <v>390</v>
       </c>
       <c r="F96" s="7"/>
       <c r="G96" s="7"/>
@@ -27443,20 +27466,20 @@
       <c r="X96" s="7"/>
     </row>
     <row r="97" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="8">
-        <v>46297</v>
-      </c>
-      <c r="B97" s="7" t="s">
+      <c r="A97" s="10">
+        <v>46275</v>
+      </c>
+      <c r="B97" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="C97" s="7" t="s">
-        <v>426</v>
-      </c>
-      <c r="D97" s="9">
-        <v>70000</v>
-      </c>
-      <c r="E97" s="8" t="s">
-        <v>434</v>
+      <c r="C97" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="D97" s="12">
+        <v>33140</v>
+      </c>
+      <c r="E97" s="11" t="s">
+        <v>277</v>
       </c>
       <c r="F97" s="7"/>
       <c r="G97" s="7"/>
@@ -27480,19 +27503,19 @@
     </row>
     <row r="98" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="8">
-        <v>46297</v>
+        <v>46295</v>
       </c>
       <c r="B98" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>427</v>
+        <v>420</v>
       </c>
       <c r="D98" s="9">
-        <v>30000</v>
+        <v>45000</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>435</v>
+        <v>422</v>
       </c>
       <c r="F98" s="7"/>
       <c r="G98" s="7"/>
@@ -27516,19 +27539,19 @@
     </row>
     <row r="99" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8">
-        <v>46299</v>
+        <v>46286</v>
       </c>
       <c r="B99" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D99" s="9">
-        <v>20000</v>
+        <v>80000</v>
       </c>
       <c r="E99" s="7" t="s">
-        <v>373</v>
+        <v>393</v>
       </c>
       <c r="F99" s="7"/>
       <c r="G99" s="7"/>
@@ -27552,19 +27575,19 @@
     </row>
     <row r="100" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="8">
-        <v>46299</v>
+        <v>46292</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>304</v>
+        <v>401</v>
       </c>
       <c r="D100" s="9">
         <v>30000</v>
       </c>
       <c r="E100" s="7" t="s">
-        <v>431</v>
+        <v>405</v>
       </c>
       <c r="F100" s="7"/>
       <c r="G100" s="7"/>
@@ -27588,19 +27611,19 @@
     </row>
     <row r="101" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="8">
-        <v>46300</v>
+        <v>46290</v>
       </c>
       <c r="B101" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>440</v>
+        <v>396</v>
       </c>
       <c r="D101" s="9">
-        <v>40000</v>
+        <v>54240</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>450</v>
+        <v>397</v>
       </c>
       <c r="F101" s="7"/>
       <c r="G101" s="7"/>
@@ -27624,19 +27647,19 @@
     </row>
     <row r="102" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="8">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="D102" s="9">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="F102" s="7"/>
       <c r="G102" s="7"/>
@@ -27660,19 +27683,19 @@
     </row>
     <row r="103" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="8">
-        <v>46300</v>
+        <v>46279</v>
       </c>
       <c r="B103" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C103" s="7" t="s">
-        <v>429</v>
+        <v>302</v>
       </c>
       <c r="D103" s="9">
-        <v>25000</v>
+        <v>36050</v>
       </c>
       <c r="E103" s="7" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="F103" s="7"/>
       <c r="G103" s="7"/>
@@ -27696,19 +27719,19 @@
     </row>
     <row r="104" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="8">
-        <v>46300</v>
+        <v>46270</v>
       </c>
       <c r="B104" s="7" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="C104" s="7" t="s">
-        <v>430</v>
+        <v>265</v>
       </c>
       <c r="D104" s="9">
         <v>50000</v>
       </c>
       <c r="E104" s="7" t="s">
-        <v>432</v>
+        <v>266</v>
       </c>
       <c r="F104" s="7"/>
       <c r="G104" s="7"/>
@@ -27732,19 +27755,19 @@
     </row>
     <row r="105" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="8">
-        <v>46300</v>
+        <v>46280</v>
       </c>
       <c r="B105" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>428</v>
+        <v>308</v>
       </c>
       <c r="D105" s="9">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="E105" s="7" t="s">
-        <v>436</v>
+        <v>322</v>
       </c>
       <c r="F105" s="7"/>
       <c r="G105" s="7"/>
@@ -27768,19 +27791,19 @@
     </row>
     <row r="106" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="8">
-        <v>46301</v>
+        <v>46285</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>447</v>
+        <v>364</v>
       </c>
       <c r="D106" s="9">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>255</v>
+        <v>376</v>
       </c>
       <c r="F106" s="7"/>
       <c r="G106" s="7"/>
@@ -27810,13 +27833,13 @@
         <v>243</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="D107" s="9">
         <v>20000</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>449</v>
+        <v>376</v>
       </c>
       <c r="F107" s="7"/>
       <c r="G107" s="7"/>
@@ -27840,19 +27863,19 @@
     </row>
     <row r="108" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="8">
-        <v>46301</v>
+        <v>46277</v>
       </c>
       <c r="B108" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>445</v>
+        <v>287</v>
       </c>
       <c r="D108" s="9">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="E108" s="7" t="s">
-        <v>448</v>
+        <v>290</v>
       </c>
       <c r="F108" s="7"/>
       <c r="G108" s="7"/>
@@ -27882,13 +27905,13 @@
         <v>243</v>
       </c>
       <c r="C109" s="7" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="D109" s="9">
-        <v>42000</v>
+        <v>40000</v>
       </c>
       <c r="E109" s="7" t="s">
-        <v>413</v>
+        <v>290</v>
       </c>
       <c r="F109" s="7"/>
       <c r="G109" s="7"/>
@@ -27912,19 +27935,19 @@
     </row>
     <row r="110" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="8">
-        <v>46301</v>
+        <v>46280</v>
       </c>
       <c r="B110" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C110" s="7" t="s">
-        <v>442</v>
+        <v>310</v>
       </c>
       <c r="D110" s="9">
-        <v>20000</v>
+        <v>44140</v>
       </c>
       <c r="E110" s="7" t="s">
-        <v>376</v>
+        <v>341</v>
       </c>
       <c r="F110" s="7"/>
       <c r="G110" s="7"/>
@@ -27948,19 +27971,19 @@
     </row>
     <row r="111" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="8">
-        <v>46301</v>
+        <v>46294</v>
       </c>
       <c r="B111" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C111" s="7" t="s">
-        <v>441</v>
+        <v>416</v>
       </c>
       <c r="D111" s="9">
         <v>40000</v>
       </c>
       <c r="E111" s="7" t="s">
-        <v>290</v>
+        <v>418</v>
       </c>
       <c r="F111" s="7"/>
       <c r="G111" s="7"/>
@@ -27984,19 +28007,19 @@
     </row>
     <row r="112" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="8">
-        <v>46302</v>
+        <v>46293</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>452</v>
+        <v>403</v>
       </c>
       <c r="D112" s="9">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="E112" s="7" t="s">
-        <v>454</v>
+        <v>409</v>
       </c>
       <c r="F112" s="7"/>
       <c r="G112" s="7"/>
@@ -28020,19 +28043,19 @@
     </row>
     <row r="113" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="8">
-        <v>46302</v>
+        <v>46266</v>
       </c>
       <c r="B113" s="7" t="s">
         <v>243</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>446</v>
+        <v>256</v>
       </c>
       <c r="D113" s="9">
-        <v>49050</v>
+        <v>50000</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>453</v>
+        <v>257</v>
       </c>
       <c r="F113" s="7"/>
       <c r="G113" s="7"/>
@@ -28055,10 +28078,21 @@
       <c r="X113" s="7"/>
     </row>
     <row r="114" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B114" s="7"/>
-      <c r="C114" s="7"/>
-      <c r="D114" s="9"/>
-      <c r="E114" s="7"/>
+      <c r="A114" s="8">
+        <v>46281</v>
+      </c>
+      <c r="B114" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C114" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D114" s="9">
+        <v>20000</v>
+      </c>
+      <c r="E114" s="7" t="s">
+        <v>339</v>
+      </c>
       <c r="F114" s="7"/>
       <c r="G114" s="7"/>
       <c r="H114" s="7"/>
@@ -28080,10 +28114,21 @@
       <c r="X114" s="7"/>
     </row>
     <row r="115" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B115" s="7"/>
-      <c r="C115" s="7"/>
-      <c r="D115" s="9"/>
-      <c r="E115" s="7"/>
+      <c r="A115" s="8">
+        <v>46286</v>
+      </c>
+      <c r="B115" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C115" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D115" s="9">
+        <v>10000</v>
+      </c>
+      <c r="E115" s="7" t="s">
+        <v>339</v>
+      </c>
       <c r="F115" s="7"/>
       <c r="G115" s="7"/>
       <c r="H115" s="7"/>
@@ -28105,10 +28150,21 @@
       <c r="X115" s="7"/>
     </row>
     <row r="116" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B116" s="7"/>
-      <c r="C116" s="7"/>
-      <c r="D116" s="9"/>
-      <c r="E116" s="7"/>
+      <c r="A116" s="8">
+        <v>46290</v>
+      </c>
+      <c r="B116" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C116" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="D116" s="9">
+        <v>16880</v>
+      </c>
+      <c r="E116" s="7" t="s">
+        <v>339</v>
+      </c>
       <c r="F116" s="7"/>
       <c r="G116" s="7"/>
       <c r="H116" s="7"/>
@@ -28130,9 +28186,18 @@
       <c r="X116" s="7"/>
     </row>
     <row r="117" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B117" s="7"/>
-      <c r="C117" s="7"/>
-      <c r="D117" s="9"/>
+      <c r="A117" s="8">
+        <v>46279</v>
+      </c>
+      <c r="B117" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="C117" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="D117" s="9">
+        <v>20180</v>
+      </c>
       <c r="E117" s="7"/>
       <c r="F117" s="7"/>
       <c r="G117" s="7"/>
@@ -28155,9 +28220,18 @@
       <c r="X117" s="7"/>
     </row>
     <row r="118" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B118" s="7"/>
-      <c r="C118" s="7"/>
-      <c r="D118" s="9"/>
+      <c r="A118" s="8">
+        <v>46304</v>
+      </c>
+      <c r="B118" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="D118" s="9">
+        <v>20200</v>
+      </c>
       <c r="E118" s="7"/>
       <c r="F118" s="7"/>
       <c r="G118" s="7"/>
@@ -28180,10 +28254,21 @@
       <c r="X118" s="7"/>
     </row>
     <row r="119" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B119" s="7"/>
-      <c r="C119" s="7"/>
-      <c r="D119" s="9"/>
-      <c r="E119" s="7"/>
+      <c r="A119" s="8">
+        <v>46307</v>
+      </c>
+      <c r="B119" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="D119" s="9">
+        <v>113750</v>
+      </c>
+      <c r="E119" s="7" t="s">
+        <v>461</v>
+      </c>
       <c r="F119" s="7"/>
       <c r="G119" s="7"/>
       <c r="H119" s="7"/>
@@ -39955,8 +40040,8 @@
       <c r="X589" s="7"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F113">
-    <sortCondition ref="A2:A113"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F118">
+    <sortCondition ref="E2:E118"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -40002,17 +40087,17 @@
       </c>
       <c r="B2" s="15">
         <f>'1ST TERM ACCOUNT'!AC137</f>
-        <v>60000</v>
+        <v>78000</v>
       </c>
       <c r="C2" s="15">
         <f>B2*0.7</f>
-        <v>42000</v>
+        <v>54600</v>
       </c>
       <c r="D2" s="15"/>
       <c r="E2" s="16"/>
       <c r="F2" s="15">
         <f>$C$2-D2</f>
-        <v>42000</v>
+        <v>54600</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -40028,7 +40113,7 @@
       <c r="E3" s="16"/>
       <c r="F3" s="15">
         <f>$C$2-(D2+D3)</f>
-        <v>42000</v>
+        <v>54600</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -40037,14 +40122,14 @@
       </c>
       <c r="B4" s="15">
         <f>B3-B2</f>
-        <v>156000</v>
+        <v>138000</v>
       </c>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="16"/>
       <c r="F4" s="15">
         <f>$C$2-(D2+D3+D4)</f>
-        <v>42000</v>
+        <v>54600</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -40054,7 +40139,7 @@
       <c r="E5" s="16"/>
       <c r="F5" s="15">
         <f>$C$2-(D2+D3+D4+D5)</f>
-        <v>42000</v>
+        <v>54600</v>
       </c>
       <c r="H5" s="17"/>
     </row>

</xml_diff>